<commit_message>
model added : ETC stochiometry modification
</commit_message>
<xml_diff>
--- a/Models/models_information.xlsx
+++ b/Models/models_information.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adam-1y9pxi6q95ggpmx\Documents\PhD\SoF1-GEM\Models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2DBCB4E-0773-4DCC-BC4B-213302FFC387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69DF3E9C-656A-475D-99D6-D810B04222DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,12 +29,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="90">
   <si>
     <t>Model Name</t>
   </si>
@@ -295,6 +298,15 @@
   </si>
   <si>
     <t>final model with corrected naming for the PAM implementation</t>
+  </si>
+  <si>
+    <t>250924_iABA974_BLG.sbml</t>
+  </si>
+  <si>
+    <t>final model with corrected ETC stochiometry</t>
+  </si>
+  <si>
+    <t>23/9/2025</t>
   </si>
 </sst>
 </file>
@@ -704,16 +716,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D34"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:D35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="52.54296875" customWidth="1"/>
+    <col min="1" max="1" width="52.5703125" customWidth="1"/>
     <col min="2" max="2" width="141" customWidth="1"/>
-    <col min="3" max="3" width="22.7265625" customWidth="1"/>
-    <col min="4" max="4" width="31.26953125" customWidth="1"/>
+    <col min="3" max="3" width="22.7109375" customWidth="1"/>
+    <col min="4" max="4" width="31.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
@@ -727,7 +739,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>12</v>
       </c>
@@ -741,7 +753,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>3</v>
       </c>
@@ -755,7 +767,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>4</v>
       </c>
@@ -769,7 +781,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>19</v>
       </c>
@@ -783,7 +795,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>8</v>
       </c>
@@ -797,7 +809,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>22</v>
       </c>
@@ -811,7 +823,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>23</v>
       </c>
@@ -825,7 +837,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>25</v>
       </c>
@@ -839,7 +851,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>27</v>
       </c>
@@ -853,7 +865,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>29</v>
       </c>
@@ -867,7 +879,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
         <v>31</v>
       </c>
@@ -881,7 +893,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
         <v>34</v>
       </c>
@@ -895,7 +907,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>36</v>
       </c>
@@ -909,7 +921,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>38</v>
       </c>
@@ -923,7 +935,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>40</v>
       </c>
@@ -937,7 +949,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
         <v>43</v>
       </c>
@@ -951,7 +963,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
         <v>46</v>
       </c>
@@ -965,7 +977,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
         <v>48</v>
       </c>
@@ -979,7 +991,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>50</v>
       </c>
@@ -993,7 +1005,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
         <v>53</v>
       </c>
@@ -1007,7 +1019,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>55</v>
       </c>
@@ -1021,7 +1033,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>58</v>
       </c>
@@ -1035,7 +1047,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
         <v>61</v>
       </c>
@@ -1049,7 +1061,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
         <v>63</v>
       </c>
@@ -1063,7 +1075,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>65</v>
       </c>
@@ -1077,7 +1089,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
         <v>68</v>
       </c>
@@ -1091,7 +1103,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
         <v>71</v>
       </c>
@@ -1105,7 +1117,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
         <v>74</v>
       </c>
@@ -1119,7 +1131,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
         <v>76</v>
       </c>
@@ -1133,7 +1145,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
         <v>78</v>
       </c>
@@ -1147,7 +1159,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
         <v>81</v>
       </c>
@@ -1159,7 +1171,7 @@
       </c>
       <c r="D32" s="1"/>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="9" t="s">
         <v>83</v>
       </c>
@@ -1171,7 +1183,7 @@
       </c>
       <c r="D33" s="9"/>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
         <v>85</v>
       </c>
@@ -1182,6 +1194,18 @@
         <v>45877</v>
       </c>
       <c r="D34" s="1"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A35" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D35" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
simulated vs experimental growth code
</commit_message>
<xml_diff>
--- a/Models/models_information.xlsx
+++ b/Models/models_information.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adam-1y9pxi6q95ggpmx\Documents\PhD\SoF1-GEM\Models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69DF3E9C-656A-475D-99D6-D810B04222DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF35BB5D-7877-490B-BB34-AFDCD73DF7C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -303,10 +303,10 @@
     <t>250924_iABA974_BLG.sbml</t>
   </si>
   <si>
-    <t>final model with corrected ETC stochiometry</t>
-  </si>
-  <si>
     <t>23/9/2025</t>
+  </si>
+  <si>
+    <t>final model with BLG production reaction</t>
   </si>
 </sst>
 </file>
@@ -1200,10 +1200,10 @@
         <v>87</v>
       </c>
       <c r="B35" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C35" s="4" t="s">
         <v>88</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>89</v>
       </c>
       <c r="D35" s="2"/>
     </row>

</xml_diff>

<commit_message>
NGAM_GAM optimizer output added
</commit_message>
<xml_diff>
--- a/Models/models_information.xlsx
+++ b/Models/models_information.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adam-1y9pxi6q95ggpmx\Documents\PhD\SoF1-GEM\Models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF35BB5D-7877-490B-BB34-AFDCD73DF7C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05274C4F-9C89-4463-9597-FB74615A8729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3795" yWindow="2085" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="93">
   <si>
     <t>Model Name</t>
   </si>
@@ -307,6 +307,15 @@
   </si>
   <si>
     <t>final model with BLG production reaction</t>
+  </si>
+  <si>
+    <t>251125_iABA974.sbml</t>
+  </si>
+  <si>
+    <t>250303_hydrogenases_completed with updated NGAM and GAM</t>
+  </si>
+  <si>
+    <t>25/11/2025</t>
   </si>
 </sst>
 </file>
@@ -352,7 +361,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -403,11 +412,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -436,6 +456,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -716,7 +739,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.5703125" customWidth="1"/>
@@ -1207,6 +1230,18 @@
       </c>
       <c r="D35" s="2"/>
     </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="14" t="s">
+        <v>90</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D36" s="16"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Modified CYTHYD stochiometry model
</commit_message>
<xml_diff>
--- a/Models/models_information.xlsx
+++ b/Models/models_information.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adam-1y9pxi6q95ggpmx\Documents\PhD\SoF1-GEM\Models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05274C4F-9C89-4463-9597-FB74615A8729}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41C66194-6F56-4861-A424-B8A24AC24548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3795" yWindow="2085" windowWidth="21600" windowHeight="11175" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -312,10 +312,10 @@
     <t>251125_iABA974.sbml</t>
   </si>
   <si>
-    <t>250303_hydrogenases_completed with updated NGAM and GAM</t>
-  </si>
-  <si>
     <t>25/11/2025</t>
+  </si>
+  <si>
+    <t>250303_hydrogenases_completed with updated NGAM and GAM  and corrected stochiometry for CYTHYD</t>
   </si>
 </sst>
 </file>
@@ -1235,10 +1235,10 @@
         <v>90</v>
       </c>
       <c r="B36" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="C36" s="7" t="s">
         <v>91</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>92</v>
       </c>
       <c r="D36" s="16"/>
     </row>

</xml_diff>

<commit_message>
Addition of the NGAM GAM itterations ploting
</commit_message>
<xml_diff>
--- a/Models/models_information.xlsx
+++ b/Models/models_information.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adam-1y9pxi6q95ggpmx\Documents\PhD\SoF1-GEM\Models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41C66194-6F56-4861-A424-B8A24AC24548}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{705928E5-0828-4942-B046-74D8266E12D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="96">
   <si>
     <t>Model Name</t>
   </si>
@@ -316,6 +316,15 @@
   </si>
   <si>
     <t>250303_hydrogenases_completed with updated NGAM and GAM  and corrected stochiometry for CYTHYD</t>
+  </si>
+  <si>
+    <t>251226_iABA974_updated_ETC.sbml</t>
+  </si>
+  <si>
+    <t>final model with updated bounds of NADH5 and only MBH active</t>
+  </si>
+  <si>
+    <t>26/12/2025</t>
   </si>
 </sst>
 </file>
@@ -361,7 +370,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -423,11 +432,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -459,6 +479,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -739,7 +760,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.5703125" customWidth="1"/>
@@ -1242,6 +1263,17 @@
       </c>
       <c r="D36" s="16"/>
     </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="C37" t="s">
+        <v>95</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
feat(Scripts): add COG enhanced annotation notebook and related data files feat(Models): update models_information.xlsx with new model data
</commit_message>
<xml_diff>
--- a/Models/models_information.xlsx
+++ b/Models/models_information.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adam-1y9pxi6q95ggpmx\Documents\PhD\SoF1-GEM\Models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{705928E5-0828-4942-B046-74D8266E12D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{651BCCF9-8EEA-46DC-B001-B77953A0B3D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="98">
   <si>
     <t>Model Name</t>
   </si>
@@ -325,6 +325,12 @@
   </si>
   <si>
     <t>26/12/2025</t>
+  </si>
+  <si>
+    <t>260302_iABA974.sbml</t>
+  </si>
+  <si>
+    <t>final model with COG annotations</t>
   </si>
 </sst>
 </file>
@@ -370,7 +376,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -421,33 +427,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -478,8 +462,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -760,7 +742,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52.5703125" customWidth="1"/>
@@ -1261,18 +1243,31 @@
       <c r="C36" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="D36" s="16"/>
+      <c r="D36" s="1"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
         <v>93</v>
       </c>
-      <c r="B37" s="17" t="s">
+      <c r="B37" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C37" s="1" t="s">
         <v>95</v>
       </c>
+      <c r="D37" s="1"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="C38" s="2">
+        <v>46056</v>
+      </c>
+      <c r="D38" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>